<commit_message>
LMDI: Merge pull request #113 from folkehelseinstituttet/roar/apne-form-coding
Åpne slicingen på Legemiddel.form.coding og bump til 1.1.5 d257194d8ac9b4a6187b91a37c8a214597864d3c
</commit_message>
<xml_diff>
--- a/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
+++ b/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.4</t>
+    <t>1.1.5</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-21T06:14:41+00:00</t>
+    <t>2026-09-21T06:15:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
LMDI: Merge pull request #120 from folkehelseinstituttet/roar/icd10-slice-flere-koder
Tillat flere ICD-10-koder på Diagnose (#117) 63d6225bf914a94af0ed1c1b1393bc20dabc50ba
</commit_message>
<xml_diff>
--- a/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
+++ b/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.6</t>
+    <t>1.1.7</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-07T08:53:26+00:00</t>
+    <t>2026-10-07T09:44:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>